<commit_message>
Update documentation to ensure consistency between security and resource models
Updated the WINDTRE-GAP-ANALYSIS-COMPLETA.md file to reflect changes made to the SERVICE-RESOURCE-MODEL-W3SUITE.xlsx and SOC-RISPOSTE-PREFILTRATE-v2.xlsx files, ensuring alignment between security compliance and resource allocation documentation.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: bd83b791-fe19-4f8c-8f08-c40cf927c2eb
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Event-Id: 22f24fdd-3281-437d-b259-971647861c37
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/990d2e08-e877-47ab-86e4-4ab1ec4a5b18/bd83b791-fe19-4f8c-8f08-c40cf927c2eb/orRbN4m
</commit_message>
<xml_diff>
--- a/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE.xlsx
+++ b/docs/gara-appalto/SERVICE-RESOURCE-MODEL-W3SUITE.xlsx
@@ -397,29 +397,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U13"/>
   <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="25.83203125" customWidth="1"/>
-    <col min="5" max="5" width="25.83203125" customWidth="1"/>
-    <col min="6" max="6" width="25.83203125" customWidth="1"/>
-    <col min="7" max="7" width="25.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-    <col min="9" max="9" width="25.83203125" customWidth="1"/>
-    <col min="10" max="10" width="25.83203125" customWidth="1"/>
-    <col min="11" max="11" width="25.83203125" customWidth="1"/>
-    <col min="12" max="12" width="25.83203125" customWidth="1"/>
-    <col min="13" max="13" width="25.83203125" customWidth="1"/>
-    <col min="14" max="14" width="25.83203125" customWidth="1"/>
-    <col min="15" max="15" width="25.83203125" customWidth="1"/>
-    <col min="16" max="16" width="25.83203125" customWidth="1"/>
-    <col min="17" max="17" width="25.83203125" customWidth="1"/>
-    <col min="18" max="18" width="25.83203125" customWidth="1"/>
-    <col min="19" max="19" width="25.83203125" customWidth="1"/>
-    <col min="20" max="20" width="25.83203125" customWidth="1"/>
-    <col min="21" max="21" width="25.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="28.83203125" customWidth="1"/>
+    <col min="5" max="5" width="28.83203125" customWidth="1"/>
+    <col min="6" max="6" width="28.83203125" customWidth="1"/>
+    <col min="7" max="7" width="28.83203125" customWidth="1"/>
+    <col min="8" max="8" width="28.83203125" customWidth="1"/>
+    <col min="9" max="9" width="28.83203125" customWidth="1"/>
+    <col min="10" max="10" width="28.83203125" customWidth="1"/>
+    <col min="11" max="11" width="28.83203125" customWidth="1"/>
+    <col min="12" max="12" width="28.83203125" customWidth="1"/>
+    <col min="13" max="13" width="28.83203125" customWidth="1"/>
+    <col min="14" max="14" width="28.83203125" customWidth="1"/>
+    <col min="15" max="15" width="28.83203125" customWidth="1"/>
+    <col min="16" max="16" width="28.83203125" customWidth="1"/>
+    <col min="17" max="17" width="28.83203125" customWidth="1"/>
+    <col min="18" max="18" width="28.83203125" customWidth="1"/>
+    <col min="19" max="19" width="28.83203125" customWidth="1"/>
+    <col min="20" max="20" width="28.83203125" customWidth="1"/>
+    <col min="21" max="21" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,7 +513,7 @@
         <v>Backend Node.js</v>
       </c>
       <c r="I2" t="str">
-        <v>Node.js 20 LTS containerized</v>
+        <v>Node.js 20 LTS con Express.js</v>
       </c>
       <c r="J2" t="str">
         <v>3</v>
@@ -643,7 +643,7 @@
         <v>Nginx Reverse Proxy</v>
       </c>
       <c r="I4" t="str">
-        <v>Nginx with TLS termination</v>
+        <v>Nginx con TLS 1.3 termination</v>
       </c>
       <c r="J4" t="str">
         <v>2</v>
@@ -693,7 +693,7 @@
         <v>HA</v>
       </c>
       <c r="D5" t="str">
-        <v>DATABASE LAYER</v>
+        <v>CORE PLATFORM</v>
       </c>
       <c r="E5" t="str">
         <v>Not W3 (Private Cloud)</v>
@@ -702,46 +702,46 @@
         <v>Seeweb</v>
       </c>
       <c r="G5" t="str">
-        <v>Mixed CaaS/PaaS</v>
+        <v>Multi-tenant SaaS</v>
       </c>
       <c r="H5" t="str">
-        <v>PostgreSQL Primary</v>
+        <v>Fortinet FortiGate Firewall</v>
       </c>
       <c r="I5" t="str">
-        <v>PostgreSQL 15 with streaming replication</v>
+        <v>WAF + IPS/IDS + Firewall rules</v>
       </c>
       <c r="J5" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" t="str">
-        <v>Primary-Replica</v>
+        <v>Active-Passive</v>
       </c>
       <c r="L5" t="str">
-        <v>Schema migration via Drizzle</v>
+        <v>Config update</v>
       </c>
       <c r="M5" t="str">
-        <v>Vertical scaling</v>
+        <v>N/A</v>
       </c>
       <c r="N5" t="str">
-        <v>Planned maintenance window</v>
+        <v>No outage</v>
       </c>
       <c r="O5" t="str">
-        <v>Daily full + WAL continuous</v>
+        <v>Config backup daily</v>
       </c>
       <c r="P5" t="str">
-        <v>Both (release + fault)</v>
+        <v>Restore for fault</v>
       </c>
       <c r="Q5" t="str">
-        <v>Automated failover to replica</v>
+        <v>Automated failover</v>
       </c>
       <c r="R5" t="str">
-        <v>&lt;15 min</v>
+        <v>&lt;5 min</v>
       </c>
       <c r="S5" t="str">
-        <v>&lt;5 min</v>
+        <v>0</v>
       </c>
       <c r="T5" t="str">
-        <v>Vendor</v>
+        <v>Seeweb (managed)</v>
       </c>
       <c r="U5" t="str">
         <v>Included in SaaS subscription</v>
@@ -758,7 +758,7 @@
         <v>HA</v>
       </c>
       <c r="D6" t="str">
-        <v>DATABASE LAYER</v>
+        <v>CORE PLATFORM</v>
       </c>
       <c r="E6" t="str">
         <v>Not W3 (Private Cloud)</v>
@@ -767,43 +767,43 @@
         <v>Seeweb</v>
       </c>
       <c r="G6" t="str">
-        <v>Mixed CaaS/PaaS</v>
+        <v>Multi-tenant SaaS</v>
       </c>
       <c r="H6" t="str">
-        <v>PostgreSQL Replica</v>
+        <v>Identity &amp; Auth Service</v>
       </c>
       <c r="I6" t="str">
-        <v>PostgreSQL 15 read replica</v>
+        <v>OAuth2/OIDC + JWT + RBAC engine</v>
       </c>
       <c r="J6" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K6" t="str">
-        <v>Standby</v>
+        <v>Multi-zone</v>
       </c>
       <c r="L6" t="str">
-        <v>Sync from Primary</v>
+        <v>GitOps deploy</v>
       </c>
       <c r="M6" t="str">
-        <v>Horizontal scaling (add replicas)</v>
+        <v>Horizontal scaling</v>
       </c>
       <c r="N6" t="str">
         <v>No outage</v>
       </c>
       <c r="O6" t="str">
-        <v>Inherited from Primary</v>
+        <v>N/A (stateless, keys in DB)</v>
       </c>
       <c r="P6" t="str">
-        <v>Read queries + failover</v>
+        <v>N/A</v>
       </c>
       <c r="Q6" t="str">
-        <v>Promote to Primary</v>
+        <v>Automated by Proxmox HA</v>
       </c>
       <c r="R6" t="str">
         <v>&lt;5 min</v>
       </c>
       <c r="S6" t="str">
-        <v>&lt;5 min</v>
+        <v>0</v>
       </c>
       <c r="T6" t="str">
         <v>Vendor</v>
@@ -823,7 +823,7 @@
         <v>HA</v>
       </c>
       <c r="D7" t="str">
-        <v>DATABASE LAYER</v>
+        <v>CORE PLATFORM</v>
       </c>
       <c r="E7" t="str">
         <v>Not W3 (Private Cloud)</v>
@@ -832,46 +832,46 @@
         <v>Seeweb</v>
       </c>
       <c r="G7" t="str">
-        <v>Mixed CaaS/PaaS</v>
+        <v>Multi-tenant SaaS</v>
       </c>
       <c r="H7" t="str">
-        <v>Ceph Storage</v>
+        <v>Audit Logging Service</v>
       </c>
       <c r="I7" t="str">
-        <v>Ceph distributed storage for persistence</v>
+        <v>Structured JSON logs + PostgreSQL audit tables</v>
       </c>
       <c r="J7" t="str">
-        <v>3+</v>
+        <v>2</v>
       </c>
       <c r="K7" t="str">
-        <v>Multi-node replicated</v>
+        <v>Active-Active</v>
       </c>
       <c r="L7" t="str">
-        <v>Rolling upgrade</v>
+        <v>GitOps deploy</v>
       </c>
       <c r="M7" t="str">
-        <v>Add storage nodes</v>
+        <v>Horizontal scaling</v>
       </c>
       <c r="N7" t="str">
         <v>No outage</v>
       </c>
       <c r="O7" t="str">
-        <v>Offsite weekly</v>
+        <v>Logs retention 90 days</v>
       </c>
       <c r="P7" t="str">
-        <v>Disaster recovery</v>
+        <v>Compliance + forensics</v>
       </c>
       <c r="Q7" t="str">
-        <v>Automated by Ceph</v>
+        <v>Automated by Proxmox HA</v>
       </c>
       <c r="R7" t="str">
-        <v>&lt;1 hour</v>
+        <v>&lt;5 min</v>
       </c>
       <c r="S7" t="str">
-        <v>&lt;5 min</v>
+        <v>&lt;1 min</v>
       </c>
       <c r="T7" t="str">
-        <v>Vendor (Seeweb managed)</v>
+        <v>Vendor</v>
       </c>
       <c r="U7" t="str">
         <v>Included in SaaS subscription</v>
@@ -882,64 +882,64 @@
         <v>PROD</v>
       </c>
       <c r="B8" t="str">
-        <v>99.5%</v>
+        <v>99.9%</v>
       </c>
       <c r="C8" t="str">
         <v>HA</v>
       </c>
       <c r="D8" t="str">
-        <v>AI SERVICES</v>
+        <v>DATABASE LAYER</v>
       </c>
       <c r="E8" t="str">
-        <v>Not W3 (Public Cloud Tenant)</v>
+        <v>Not W3 (Private Cloud)</v>
       </c>
       <c r="F8" t="str">
-        <v>OpenAI</v>
+        <v>Seeweb</v>
       </c>
       <c r="G8" t="str">
-        <v>Multi-tenant SaaS</v>
+        <v>Mixed CaaS/PaaS</v>
       </c>
       <c r="H8" t="str">
-        <v>OpenAI GPT API</v>
+        <v>PostgreSQL Primary</v>
       </c>
       <c r="I8" t="str">
-        <v>OpenAI API (GPT-4, GPT-3.5)</v>
+        <v>PostgreSQL 15 con streaming replication</v>
       </c>
       <c r="J8" t="str">
-        <v>N/A (SaaS)</v>
+        <v>1</v>
       </c>
       <c r="K8" t="str">
-        <v>Cloud-managed</v>
+        <v>Primary-Replica</v>
       </c>
       <c r="L8" t="str">
-        <v>API version pinning</v>
+        <v>Schema migration via Drizzle ORM</v>
       </c>
       <c r="M8" t="str">
-        <v>Rate limit management</v>
+        <v>Vertical scaling</v>
       </c>
       <c r="N8" t="str">
-        <v>No outage</v>
+        <v>Planned maintenance window</v>
       </c>
       <c r="O8" t="str">
-        <v>N/A (external SaaS)</v>
+        <v>Daily full + WAL continuous</v>
       </c>
       <c r="P8" t="str">
-        <v>N/A</v>
+        <v>Both (release + fault)</v>
       </c>
       <c r="Q8" t="str">
-        <v>Fallback to alternative model</v>
+        <v>Automated failover to replica</v>
       </c>
       <c r="R8" t="str">
+        <v>&lt;15 min</v>
+      </c>
+      <c r="S8" t="str">
         <v>&lt;5 min</v>
       </c>
-      <c r="S8" t="str">
-        <v>0</v>
-      </c>
       <c r="T8" t="str">
-        <v>OpenAI (external)</v>
+        <v>Vendor</v>
       </c>
       <c r="U8" t="str">
-        <v>Pay-per-use (tokens)</v>
+        <v>Included in SaaS subscription</v>
       </c>
     </row>
     <row r="9">
@@ -953,7 +953,7 @@
         <v>HA</v>
       </c>
       <c r="D9" t="str">
-        <v>AI SERVICES</v>
+        <v>DATABASE LAYER</v>
       </c>
       <c r="E9" t="str">
         <v>Not W3 (Private Cloud)</v>
@@ -962,54 +962,314 @@
         <v>Seeweb</v>
       </c>
       <c r="G9" t="str">
-        <v>Multi-tenant SaaS</v>
+        <v>Mixed CaaS/PaaS</v>
       </c>
       <c r="H9" t="str">
-        <v>AI Gateway (MCP)</v>
+        <v>PostgreSQL Replica</v>
       </c>
       <c r="I9" t="str">
-        <v>Node.js MCP Gateway for AI routing</v>
+        <v>PostgreSQL 15 read replica + failover target</v>
       </c>
       <c r="J9" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" t="str">
-        <v>Active-Active</v>
+        <v>Standby</v>
       </c>
       <c r="L9" t="str">
-        <v>GitOps incremental deploy</v>
+        <v>Sync from Primary</v>
       </c>
       <c r="M9" t="str">
-        <v>Horizontal scaling</v>
+        <v>Horizontal scaling (add replicas)</v>
       </c>
       <c r="N9" t="str">
         <v>No outage</v>
       </c>
       <c r="O9" t="str">
-        <v>N/A (stateless)</v>
+        <v>Inherited from Primary</v>
       </c>
       <c r="P9" t="str">
-        <v>N/A</v>
+        <v>Read queries + failover</v>
       </c>
       <c r="Q9" t="str">
-        <v>Automated by Proxmox HA</v>
+        <v>Promote to Primary</v>
       </c>
       <c r="R9" t="str">
         <v>&lt;5 min</v>
       </c>
       <c r="S9" t="str">
-        <v>0</v>
+        <v>&lt;5 min</v>
       </c>
       <c r="T9" t="str">
         <v>Vendor</v>
       </c>
       <c r="U9" t="str">
+        <v>Included in SaaS subscription</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>PROD</v>
+      </c>
+      <c r="B10" t="str">
+        <v>99.9%</v>
+      </c>
+      <c r="C10" t="str">
+        <v>HA</v>
+      </c>
+      <c r="D10" t="str">
+        <v>DATABASE LAYER</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Not W3 (Private Cloud)</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Seeweb</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Mixed CaaS/PaaS</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Ceph Storage</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Ceph distributed storage per persistenza</v>
+      </c>
+      <c r="J10" t="str">
+        <v>3+</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Multi-node replicated</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Rolling upgrade</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Add storage nodes</v>
+      </c>
+      <c r="N10" t="str">
+        <v>No outage</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Offsite weekly</v>
+      </c>
+      <c r="P10" t="str">
+        <v>Disaster recovery</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>Automated by Ceph</v>
+      </c>
+      <c r="R10" t="str">
+        <v>&lt;1 hour</v>
+      </c>
+      <c r="S10" t="str">
+        <v>&lt;5 min</v>
+      </c>
+      <c r="T10" t="str">
+        <v>Seeweb (managed)</v>
+      </c>
+      <c r="U10" t="str">
+        <v>Included in SaaS subscription</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>PROD</v>
+      </c>
+      <c r="B11" t="str">
+        <v>99.9%</v>
+      </c>
+      <c r="C11" t="str">
+        <v>HA</v>
+      </c>
+      <c r="D11" t="str">
+        <v>DATABASE LAYER</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Not W3 (Private Cloud)</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Seeweb</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Mixed CaaS/PaaS</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Secret Manager (predisposto)</v>
+      </c>
+      <c r="I11" t="str">
+        <v>AES-256-GCM encryption + env vars (Vault integrabile)</v>
+      </c>
+      <c r="J11" t="str">
+        <v>1</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Integrated</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Config update</v>
+      </c>
+      <c r="M11" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N11" t="str">
+        <v>No outage</v>
+      </c>
+      <c r="O11" t="str">
+        <v>Encrypted backup daily</v>
+      </c>
+      <c r="P11" t="str">
+        <v>Recovery</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>Manual restore</v>
+      </c>
+      <c r="R11" t="str">
+        <v>&lt;30 min</v>
+      </c>
+      <c r="S11" t="str">
+        <v>&lt;24 hours</v>
+      </c>
+      <c r="T11" t="str">
+        <v>Vendor</v>
+      </c>
+      <c r="U11" t="str">
+        <v>Included in SaaS subscription</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>PROD</v>
+      </c>
+      <c r="B12" t="str">
+        <v>99.5%</v>
+      </c>
+      <c r="C12" t="str">
+        <v>HA</v>
+      </c>
+      <c r="D12" t="str">
+        <v>AI SERVICES</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Not W3 (Public Cloud Tenant)</v>
+      </c>
+      <c r="F12" t="str">
+        <v>OpenAI</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Multi-tenant SaaS</v>
+      </c>
+      <c r="H12" t="str">
+        <v>OpenAI GPT API</v>
+      </c>
+      <c r="I12" t="str">
+        <v>OpenAI API (GPT-4, GPT-3.5-turbo)</v>
+      </c>
+      <c r="J12" t="str">
+        <v>N/A (SaaS esterno)</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Cloud-managed by OpenAI</v>
+      </c>
+      <c r="L12" t="str">
+        <v>API version pinning</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Rate limit management</v>
+      </c>
+      <c r="N12" t="str">
+        <v>No outage</v>
+      </c>
+      <c r="O12" t="str">
+        <v>N/A (external SaaS)</v>
+      </c>
+      <c r="P12" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>Fallback to alternative model</v>
+      </c>
+      <c r="R12" t="str">
+        <v>&lt;5 min</v>
+      </c>
+      <c r="S12" t="str">
+        <v>0</v>
+      </c>
+      <c r="T12" t="str">
+        <v>OpenAI (external)</v>
+      </c>
+      <c r="U12" t="str">
+        <v>Pay-per-use (tokens)</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>PROD</v>
+      </c>
+      <c r="B13" t="str">
+        <v>99.9%</v>
+      </c>
+      <c r="C13" t="str">
+        <v>HA</v>
+      </c>
+      <c r="D13" t="str">
+        <v>AI SERVICES</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Not W3 (Private Cloud)</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Seeweb</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Multi-tenant SaaS</v>
+      </c>
+      <c r="H13" t="str">
+        <v>AI Gateway (MCP)</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Node.js MCP Gateway per AI routing e orchestrazione</v>
+      </c>
+      <c r="J13" t="str">
+        <v>2</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Active-Active</v>
+      </c>
+      <c r="L13" t="str">
+        <v>GitOps incremental deploy</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Horizontal scaling</v>
+      </c>
+      <c r="N13" t="str">
+        <v>No outage</v>
+      </c>
+      <c r="O13" t="str">
+        <v>N/A (stateless)</v>
+      </c>
+      <c r="P13" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>Automated by Proxmox HA</v>
+      </c>
+      <c r="R13" t="str">
+        <v>&lt;5 min</v>
+      </c>
+      <c r="S13" t="str">
+        <v>0</v>
+      </c>
+      <c r="T13" t="str">
+        <v>Vendor</v>
+      </c>
+      <c r="U13" t="str">
         <v>Included in SaaS subscription</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>